<commit_message>
Rev. B: 18 ETNA 26 (3 sıra × 6), ultra ışık renderları, tavan planı A3 PDF
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04_Malzeme_listesi.xlsx
+++ b/04_Malzeme_listesi.xlsx
@@ -482,11 +482,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Gömme çok gözlü vitrin armatürü, 50 W, 38°, 12 sıcak + 14 beyaz göz</t>
+          <t>Gömme çok gözlü vitrin armatürü, 50 W, 25°, 12 sıcak + 14 beyaz göz</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -602,11 +602,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10 × 50 W + şerit 30 W</t>
+          <t>18 × 50 W + şerit 30 W</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>530</v>
+        <v>930</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -657,10 +657,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>300</v>
+        <v>233</v>
       </c>
       <c r="C2" t="n">
-        <v>213</v>
+        <v>138</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -675,10 +675,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>300</v>
+        <v>233</v>
       </c>
       <c r="C3" t="n">
-        <v>517</v>
+        <v>365</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -689,14 +689,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E2A</t>
+          <t>E1C</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>770</v>
+        <v>233</v>
       </c>
       <c r="C4" t="n">
-        <v>213</v>
+        <v>592</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -707,14 +707,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E2B</t>
+          <t>E2A</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>770</v>
+        <v>636</v>
       </c>
       <c r="C5" t="n">
-        <v>517</v>
+        <v>138</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -725,14 +725,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>E3A</t>
+          <t>E2B</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1240</v>
+        <v>636</v>
       </c>
       <c r="C6" t="n">
-        <v>213</v>
+        <v>365</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -743,14 +743,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>E3B</t>
+          <t>E2C</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1240</v>
+        <v>636</v>
       </c>
       <c r="C7" t="n">
-        <v>517</v>
+        <v>592</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -761,14 +761,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>E4A</t>
+          <t>E3A</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1710</v>
+        <v>1039</v>
       </c>
       <c r="C8" t="n">
-        <v>213</v>
+        <v>138</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -779,14 +779,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>E4B</t>
+          <t>E3B</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1710</v>
+        <v>1039</v>
       </c>
       <c r="C9" t="n">
-        <v>517</v>
+        <v>365</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -797,14 +797,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>E5A</t>
+          <t>E3C</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2180</v>
+        <v>1039</v>
       </c>
       <c r="C10" t="n">
-        <v>213</v>
+        <v>592</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -815,16 +815,160 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>E4A</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1441</v>
+      </c>
+      <c r="C11" t="n">
+        <v>138</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>320 × 155</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>E4B</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1441</v>
+      </c>
+      <c r="C12" t="n">
+        <v>365</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>320 × 155</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E4C</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1441</v>
+      </c>
+      <c r="C13" t="n">
+        <v>592</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>320 × 155</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>E5A</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C14" t="n">
+        <v>138</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>320 × 155</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>E5B</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>2180</v>
-      </c>
-      <c r="C11" t="n">
-        <v>517</v>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="B15" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C15" t="n">
+        <v>365</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>320 × 155</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>E5C</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C16" t="n">
+        <v>592</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>320 × 155</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>E6A</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2247</v>
+      </c>
+      <c r="C17" t="n">
+        <v>138</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>320 × 155</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>E6B</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2247</v>
+      </c>
+      <c r="C18" t="n">
+        <v>365</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>320 × 155</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>E6C</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2247</v>
+      </c>
+      <c r="C19" t="n">
+        <v>592</v>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>320 × 155</t>
         </is>

</xml_diff>